<commit_message>
Komodo Added: - Activities (1).csv - AA377396-voucher.pdf - All Indonesia.pdf - Drone Operation Guidelines \342\200\223 Komodo National Park.pdf" - Indonesia-Drone-Permit.pdf - LA_Guest_Gaya_Baru_Indah.pdf - LA_Guest_Naga_Biru.pdf - NAGA BIRU - Liability Release.pdf - Surat Pernyataan Drone_english version.docx - Z7A5569586.pdf - booking-com.png - lionair-support.png - NagaBiru-DPS-LBJ.pdf Modified: - Activities.csv - Diving.code-workspace - Format.xlsm - trip-proposals.md - Scuba_Log.xlsx
</commit_message>
<xml_diff>
--- a/Scuba_Log.xlsx
+++ b/Scuba_Log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Akseldkw/Desktop/Aksel/Diving/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F372605D-2473-4040-9B69-FBF8E2050CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AE7D01-8ECE-0B45-BEC7-67A278813DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="28460" windowHeight="17680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3360" yWindow="760" windowWidth="28460" windowHeight="23780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2630" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2740" uniqueCount="557">
   <si>
     <t>Dive Number</t>
   </si>
@@ -1448,21 +1448,228 @@
     <t>0 days 02:55:35</t>
   </si>
   <si>
+    <t xml:space="preserve">Lionfish hunt dive. Not super noteworthy, didn't see a ton of them </t>
+  </si>
+  <si>
+    <t>Shark Point</t>
+  </si>
+  <si>
     <t>0 days 16:04:55</t>
   </si>
   <si>
+    <t xml:space="preserve">Very cool dive. Grouper was swimming me with the whole time, tried to get a shot and feed off but the sharks were way too close to pull it off. Got a nice video of me and the grouper hanging out </t>
+  </si>
+  <si>
     <t>0 days 01:36:41</t>
   </si>
   <si>
+    <t xml:space="preserve">Things got a little hairy here. I decided to risk it on a couple of lionfish shots to feed the friendly grouper. The first one was stolen by a reef shark, the second one got away but didn't stop the reef sharks from swarming me </t>
+  </si>
+  <si>
     <t>0 days 03:19:02</t>
   </si>
   <si>
+    <t>Hat Key</t>
+  </si>
+  <si>
     <t>0 days 16:22:19</t>
   </si>
   <si>
+    <t>Back to the south near hat key for lionfish hunts, Dan took us super far south this time to find virgin reef. I was really on my game this dive - probably shot nearly half of the lionfish our group took the whole dive. Nearly ran out of air at the end with Axel</t>
+  </si>
+  <si>
     <t>0 days 01:02:37</t>
   </si>
   <si>
+    <t>Sweet final dive, another lionfish hunt. Tom and I took 3 lionfish out of this one hole in a great feat of teamwork. Bit slower than the first dive, but very fun nonetheless</t>
+  </si>
+  <si>
+    <t>Labuan Haji</t>
+  </si>
+  <si>
+    <t>Mojo Island</t>
+  </si>
+  <si>
+    <t>Very clear and calm</t>
+  </si>
+  <si>
+    <t>No current</t>
+  </si>
+  <si>
+    <t>EANx (+1)</t>
+  </si>
+  <si>
+    <t>63 days 13:48:19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First dive of the trip. Shallow wall, beautiful coral. We swam over the eel snakes </t>
+  </si>
+  <si>
+    <t>Clear, night</t>
+  </si>
+  <si>
+    <t>0 days 03:09:48</t>
+  </si>
+  <si>
+    <t>Night dive on same reef from the morning</t>
+  </si>
+  <si>
+    <t>Tik Selah Bay</t>
+  </si>
+  <si>
+    <t>Teluk Saleh</t>
+  </si>
+  <si>
+    <t>Sunrise</t>
+  </si>
+  <si>
+    <t>Strong current</t>
+  </si>
+  <si>
+    <t>0 days 00:23:04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whale shark dive! It was a bit manufactured and depressing that the shark was just getting fed </t>
+  </si>
+  <si>
+    <t>Sumbawa Wall</t>
+  </si>
+  <si>
+    <t>Pulau Satonda</t>
+  </si>
+  <si>
+    <t>0 days 07:05:13</t>
+  </si>
+  <si>
+    <t>Very cool dive. The dive ended early because Whitney and mom ran out of air, but was very cool to get swept by current over shallow reef. There was a pier</t>
+  </si>
+  <si>
+    <t>Satondo</t>
+  </si>
+  <si>
+    <t>Raining</t>
+  </si>
+  <si>
+    <t>0 days 02:50:52</t>
+  </si>
+  <si>
+    <t>Night dive with Mom. Saw crocodile fish, big cuttlefish</t>
+  </si>
+  <si>
+    <t>Tikno Reef</t>
+  </si>
+  <si>
+    <t>Sangiang</t>
+  </si>
+  <si>
+    <t>Overcast</t>
+  </si>
+  <si>
+    <t>Warm</t>
+  </si>
+  <si>
+    <t>0 days 14:53:23</t>
+  </si>
+  <si>
+    <t>Pretty boring, looked too long at the muck. Mom and I went up early, was cool to use the SMB</t>
+  </si>
+  <si>
+    <t>Lighthouse</t>
+  </si>
+  <si>
+    <t>Strong current, variable temperature</t>
+  </si>
+  <si>
+    <t>0 days 03:32:21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very cool dive. Got some excellent footage of corals </t>
+  </si>
+  <si>
+    <t>Hot Rocks</t>
+  </si>
+  <si>
+    <t>Turbid, decent current, bits of cold</t>
+  </si>
+  <si>
+    <t>0 days 15:41:06</t>
+  </si>
+  <si>
+    <t>Volcanic warm water bubbling up from the sandy bottom. Saw lots of soft corals, anemones, schooling fish. At the end of dive, I came across a mantis shrimp. Wasn't able to get it to hit my coral</t>
+  </si>
+  <si>
+    <t>Gili Banta Bay</t>
+  </si>
+  <si>
+    <t>Gili Banta Island</t>
+  </si>
+  <si>
+    <t>Sunny</t>
+  </si>
+  <si>
+    <t>0 days 03:34:43</t>
+  </si>
+  <si>
+    <t>Cool dive, very strong current at the end. We spent a lot of time fighting the current</t>
+  </si>
+  <si>
+    <t>Batu Monco</t>
+  </si>
+  <si>
+    <t>Komodo</t>
+  </si>
+  <si>
+    <t>0 days 03:12:02</t>
+  </si>
+  <si>
+    <t>Best dive yet. Tons of fish, felt like a little fishtank. Mom accidentally knocked my watch off, and I lost it at the end of the dive (luckily recovered)</t>
+  </si>
+  <si>
+    <t>The Shotgun</t>
+  </si>
+  <si>
+    <t>Warm, windy</t>
+  </si>
+  <si>
+    <t>Strong current, very active thermocline</t>
+  </si>
+  <si>
+    <t>0 days 14:57:27</t>
+  </si>
+  <si>
+    <t>Sickest dive yet. Dropped in on a huge school of fish. From there, current swept us over the shotgun and big hole. Came up at the other end, saw GT</t>
+  </si>
+  <si>
+    <t>Tatawa Besar</t>
+  </si>
+  <si>
+    <t>Chill current</t>
+  </si>
+  <si>
+    <t>0 days 02:48:58</t>
+  </si>
+  <si>
+    <t>Cool dive, saw turtles and reef sharks</t>
+  </si>
+  <si>
+    <t>Mawan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warm </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very strong current </t>
+  </si>
+  <si>
+    <t>0 days 01:52:22</t>
+  </si>
+  <si>
+    <t>Manta dive!! So many mantas, just unreal. Manta came very close to me. Saw a blacktip reef shark as well</t>
+  </si>
+  <si>
+    <t>0 days 15:39:35</t>
+  </si>
+  <si>
     <t xml:space="preserve">First Huracan dive. DM was named Eric, really great dive. Saw reef shark, tarpon, snapper, schools of fish. Drift dive, wall started at 30ft and continued into the abyss to ~200 ft. Shot 3 lionfish and missed 2 more, saw shark right after shooting lionfish which spooked me a bit. </t>
   </si>
   <si>
@@ -1475,25 +1682,16 @@
     <t>Wall dive, buddied with mom. Saw no lionfish again! 3 turtles, reef sharkkd</t>
   </si>
   <si>
-    <t>Shark Point</t>
-  </si>
-  <si>
-    <t>Hat Key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lionfish hunt dive. Not super noteworthy, didn't see a ton of them </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very cool dive. Grouper was swimming me with the whole time, tried to get a shot and feed off but the sharks were way too close to pull it off. Got a nice video of me and the grouper hanging out </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Things got a little hairy here. I decided to risk it on a couple of lionfish shots to feed the friendly grouper. The first one was stolen by a reef shark, the second one got away but didn't stop the reef sharks from swarming me </t>
-  </si>
-  <si>
-    <t>Sweet final dive, another lionfish hunt. Tom and I took 3 lionfish out of this one hole in a great feat of teamwork. Bit slower than the first dive, but very fun nonetheless</t>
-  </si>
-  <si>
-    <t>Back to the south near hat key for lionfish hunts, Dan took us super far south this time to find virgin reef. I was really on my game this dive - probably shot nearly half of the lionfish our group took the whole dive. Nearly ran out of air at the end with Axel</t>
+    <t>Manta Alley</t>
+  </si>
+  <si>
+    <t>Early morning, sunny</t>
+  </si>
+  <si>
+    <t>Cold</t>
+  </si>
+  <si>
+    <t>Manta dive p2. Water was much murkier and colder than the previous days. We dove down to a manta cleaning station, but were unable to see as many. The current was very strong. The water was cold enough to take my breath away for a few seconds after entering</t>
   </si>
 </sst>
 </file>
@@ -1521,7 +1719,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1558,6 +1756,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1580,7 +1784,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1609,6 +1813,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1949,7 +2156,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S188"/>
+  <dimension ref="A1:S202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" customWidth="1"/>
@@ -10712,7 +10919,7 @@
         <v>98</v>
       </c>
       <c r="R183" s="3" t="s">
-        <v>486</v>
+        <v>475</v>
       </c>
     </row>
     <row r="184" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -10726,7 +10933,7 @@
         <v>417</v>
       </c>
       <c r="D184" s="3" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="E184" s="3" t="s">
         <v>233</v>
@@ -10747,7 +10954,7 @@
         <v>61</v>
       </c>
       <c r="N184" s="3" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="P184" s="3">
         <v>81</v>
@@ -10756,7 +10963,7 @@
         <v>111</v>
       </c>
       <c r="R184" s="3" t="s">
-        <v>487</v>
+        <v>478</v>
       </c>
     </row>
     <row r="185" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -10791,7 +10998,7 @@
         <v>62</v>
       </c>
       <c r="N185" s="3" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="P185" s="3">
         <v>75</v>
@@ -10800,7 +11007,7 @@
         <v>94</v>
       </c>
       <c r="R185" s="3" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
     </row>
     <row r="186" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -10835,7 +11042,7 @@
         <v>68</v>
       </c>
       <c r="N186" s="3" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="P186" s="3">
         <v>56</v>
@@ -10844,7 +11051,7 @@
         <v>83</v>
       </c>
       <c r="R186" s="3" t="s">
-        <v>486</v>
+        <v>475</v>
       </c>
     </row>
     <row r="187" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -10858,7 +11065,7 @@
         <v>417</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="E187" s="3" t="s">
         <v>179</v>
@@ -10879,7 +11086,7 @@
         <v>66</v>
       </c>
       <c r="N187" s="3" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="P187" s="3">
         <v>84</v>
@@ -10888,7 +11095,7 @@
         <v>110</v>
       </c>
       <c r="R187" s="3" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
     </row>
     <row r="188" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -10923,7 +11130,7 @@
         <v>72</v>
       </c>
       <c r="N188" s="3" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="P188" s="3">
         <v>75</v>
@@ -10932,7 +11139,737 @@
         <v>93</v>
       </c>
       <c r="R188" s="3" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="189" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A189" s="26">
+        <v>220</v>
+      </c>
+      <c r="B189" s="27">
+        <v>46159</v>
+      </c>
+      <c r="C189" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D189" s="26" t="s">
+        <v>487</v>
+      </c>
+      <c r="E189" s="26" t="s">
+        <v>488</v>
+      </c>
+      <c r="F189" s="26" t="s">
         <v>489</v>
+      </c>
+      <c r="G189" s="26" t="s">
+        <v>490</v>
+      </c>
+      <c r="H189" s="26">
+        <v>52</v>
+      </c>
+      <c r="I189" s="26">
+        <v>86</v>
+      </c>
+      <c r="J189" s="26">
+        <v>60</v>
+      </c>
+      <c r="K189" s="28">
+        <v>0.61319444444444449</v>
+      </c>
+      <c r="L189" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M189" s="26">
+        <v>61</v>
+      </c>
+      <c r="N189" s="26" t="s">
+        <v>492</v>
+      </c>
+      <c r="P189" s="26">
+        <v>77</v>
+      </c>
+      <c r="Q189" s="26">
+        <v>99</v>
+      </c>
+      <c r="R189" s="26" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="190" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A190" s="26">
+        <v>221</v>
+      </c>
+      <c r="B190" s="27">
+        <v>46159</v>
+      </c>
+      <c r="C190" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D190" s="26" t="s">
+        <v>487</v>
+      </c>
+      <c r="E190" s="26" t="s">
+        <v>488</v>
+      </c>
+      <c r="F190" s="26" t="s">
+        <v>494</v>
+      </c>
+      <c r="G190" s="26" t="s">
+        <v>490</v>
+      </c>
+      <c r="H190" s="26">
+        <v>51</v>
+      </c>
+      <c r="I190" s="26">
+        <v>86</v>
+      </c>
+      <c r="J190" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="K190" s="28">
+        <v>0.78680555555555554</v>
+      </c>
+      <c r="L190" s="26" t="s">
+        <v>400</v>
+      </c>
+      <c r="M190" s="26">
+        <v>65</v>
+      </c>
+      <c r="N190" s="26" t="s">
+        <v>495</v>
+      </c>
+      <c r="P190" s="26">
+        <v>66</v>
+      </c>
+      <c r="Q190" s="26">
+        <v>85</v>
+      </c>
+      <c r="R190" s="26" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="191" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A191" s="26">
+        <v>223</v>
+      </c>
+      <c r="B191" s="27">
+        <v>46160</v>
+      </c>
+      <c r="C191" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D191" s="26" t="s">
+        <v>497</v>
+      </c>
+      <c r="E191" s="26" t="s">
+        <v>498</v>
+      </c>
+      <c r="F191" s="26" t="s">
+        <v>499</v>
+      </c>
+      <c r="G191" s="26" t="s">
+        <v>500</v>
+      </c>
+      <c r="H191" s="26">
+        <v>28</v>
+      </c>
+      <c r="I191" s="26">
+        <v>86</v>
+      </c>
+      <c r="J191" s="26">
+        <v>60</v>
+      </c>
+      <c r="K191" s="28">
+        <v>0.30902777777777779</v>
+      </c>
+      <c r="L191" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M191" s="26">
+        <v>35</v>
+      </c>
+      <c r="N191" s="26" t="s">
+        <v>501</v>
+      </c>
+      <c r="P191" s="26">
+        <v>83</v>
+      </c>
+      <c r="Q191" s="26">
+        <v>112</v>
+      </c>
+      <c r="R191" s="26" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="192" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A192" s="26">
+        <v>224</v>
+      </c>
+      <c r="B192" s="27">
+        <v>46160</v>
+      </c>
+      <c r="C192" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D192" s="26" t="s">
+        <v>503</v>
+      </c>
+      <c r="E192" s="26" t="s">
+        <v>504</v>
+      </c>
+      <c r="H192" s="26">
+        <v>86</v>
+      </c>
+      <c r="I192" s="26">
+        <v>86</v>
+      </c>
+      <c r="J192" s="26">
+        <v>60</v>
+      </c>
+      <c r="K192" s="28">
+        <v>0.62847222222222221</v>
+      </c>
+      <c r="L192" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M192" s="26">
+        <v>42</v>
+      </c>
+      <c r="N192" s="26" t="s">
+        <v>505</v>
+      </c>
+      <c r="P192" s="26">
+        <v>72</v>
+      </c>
+      <c r="Q192" s="26">
+        <v>94</v>
+      </c>
+      <c r="R192" s="26" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="193" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A193" s="26">
+        <v>225</v>
+      </c>
+      <c r="B193" s="27">
+        <v>46160</v>
+      </c>
+      <c r="C193" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D193" s="26" t="s">
+        <v>507</v>
+      </c>
+      <c r="E193" s="26" t="s">
+        <v>504</v>
+      </c>
+      <c r="F193" s="26" t="s">
+        <v>508</v>
+      </c>
+      <c r="H193" s="26">
+        <v>55</v>
+      </c>
+      <c r="I193" s="26">
+        <v>86</v>
+      </c>
+      <c r="J193" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="K193" s="28">
+        <v>0.77569444444444446</v>
+      </c>
+      <c r="L193" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M193" s="26">
+        <v>61</v>
+      </c>
+      <c r="N193" s="26" t="s">
+        <v>509</v>
+      </c>
+      <c r="P193" s="26">
+        <v>69</v>
+      </c>
+      <c r="Q193" s="26">
+        <v>87</v>
+      </c>
+      <c r="R193" s="26" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="194" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A194" s="26">
+        <v>226</v>
+      </c>
+      <c r="B194" s="27">
+        <v>46161</v>
+      </c>
+      <c r="C194" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D194" s="26" t="s">
+        <v>511</v>
+      </c>
+      <c r="E194" s="26" t="s">
+        <v>512</v>
+      </c>
+      <c r="F194" s="26" t="s">
+        <v>513</v>
+      </c>
+      <c r="G194" s="26" t="s">
+        <v>514</v>
+      </c>
+      <c r="H194" s="26">
+        <v>61</v>
+      </c>
+      <c r="I194" s="26">
+        <v>84.2</v>
+      </c>
+      <c r="J194" s="26">
+        <v>60</v>
+      </c>
+      <c r="K194" s="28">
+        <v>0.4375</v>
+      </c>
+      <c r="L194" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M194" s="26">
+        <v>52</v>
+      </c>
+      <c r="N194" s="26" t="s">
+        <v>515</v>
+      </c>
+      <c r="P194" s="26">
+        <v>74</v>
+      </c>
+      <c r="Q194" s="26">
+        <v>93</v>
+      </c>
+      <c r="R194" s="26" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="195" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A195" s="26">
+        <v>227</v>
+      </c>
+      <c r="B195" s="27">
+        <v>46161</v>
+      </c>
+      <c r="C195" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D195" s="26" t="s">
+        <v>517</v>
+      </c>
+      <c r="E195" s="26" t="s">
+        <v>512</v>
+      </c>
+      <c r="F195" s="26" t="s">
+        <v>513</v>
+      </c>
+      <c r="G195" s="26" t="s">
+        <v>518</v>
+      </c>
+      <c r="H195" s="26">
+        <v>87</v>
+      </c>
+      <c r="I195" s="26">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="J195" s="26">
+        <v>60</v>
+      </c>
+      <c r="K195" s="28">
+        <v>0.62013888888888891</v>
+      </c>
+      <c r="L195" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M195" s="26">
+        <v>55</v>
+      </c>
+      <c r="N195" s="26" t="s">
+        <v>519</v>
+      </c>
+      <c r="P195" s="26">
+        <v>73</v>
+      </c>
+      <c r="Q195" s="26">
+        <v>95</v>
+      </c>
+      <c r="R195" s="26" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="196" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A196" s="26">
+        <v>228</v>
+      </c>
+      <c r="B196" s="27">
+        <v>46162</v>
+      </c>
+      <c r="C196" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D196" s="26" t="s">
+        <v>521</v>
+      </c>
+      <c r="E196" s="26" t="s">
+        <v>512</v>
+      </c>
+      <c r="F196" s="26" t="s">
+        <v>499</v>
+      </c>
+      <c r="G196" s="26" t="s">
+        <v>522</v>
+      </c>
+      <c r="H196" s="26">
+        <v>72</v>
+      </c>
+      <c r="I196" s="26">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="J196" s="26">
+        <v>60</v>
+      </c>
+      <c r="K196" s="28">
+        <v>0.31180555555555556</v>
+      </c>
+      <c r="L196" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M196" s="26">
+        <v>63</v>
+      </c>
+      <c r="N196" s="26" t="s">
+        <v>523</v>
+      </c>
+      <c r="P196" s="26">
+        <v>67</v>
+      </c>
+      <c r="Q196" s="26">
+        <v>87</v>
+      </c>
+      <c r="R196" s="26" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="197" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A197" s="26">
+        <v>247</v>
+      </c>
+      <c r="B197" s="27">
+        <v>46162</v>
+      </c>
+      <c r="C197" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D197" s="26" t="s">
+        <v>525</v>
+      </c>
+      <c r="E197" s="26" t="s">
+        <v>526</v>
+      </c>
+      <c r="F197" s="26" t="s">
+        <v>527</v>
+      </c>
+      <c r="G197" s="26" t="s">
+        <v>500</v>
+      </c>
+      <c r="H197" s="26">
+        <v>82</v>
+      </c>
+      <c r="I197" s="26">
+        <v>82.4</v>
+      </c>
+      <c r="J197" s="26">
+        <v>80</v>
+      </c>
+      <c r="K197" s="28">
+        <v>0.50416666666666665</v>
+      </c>
+      <c r="L197" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M197" s="26">
+        <v>54</v>
+      </c>
+      <c r="N197" s="26" t="s">
+        <v>528</v>
+      </c>
+      <c r="P197" s="26">
+        <v>71</v>
+      </c>
+      <c r="Q197" s="26">
+        <v>92</v>
+      </c>
+      <c r="R197" s="26" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="198" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A198" s="26">
+        <v>248</v>
+      </c>
+      <c r="B198" s="27">
+        <v>46162</v>
+      </c>
+      <c r="C198" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D198" s="26" t="s">
+        <v>530</v>
+      </c>
+      <c r="E198" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="G198" s="26" t="s">
+        <v>490</v>
+      </c>
+      <c r="H198" s="26">
+        <v>40</v>
+      </c>
+      <c r="I198" s="26">
+        <v>86</v>
+      </c>
+      <c r="J198" s="26">
+        <v>80</v>
+      </c>
+      <c r="K198" s="28">
+        <v>0.6743055555555556</v>
+      </c>
+      <c r="L198" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M198" s="26">
+        <v>69</v>
+      </c>
+      <c r="N198" s="26" t="s">
+        <v>532</v>
+      </c>
+      <c r="P198" s="26">
+        <v>66</v>
+      </c>
+      <c r="Q198" s="26">
+        <v>107</v>
+      </c>
+      <c r="R198" s="26" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="199" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A199" s="26">
+        <v>249</v>
+      </c>
+      <c r="B199" s="27">
+        <v>46163</v>
+      </c>
+      <c r="C199" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D199" s="26" t="s">
+        <v>534</v>
+      </c>
+      <c r="E199" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F199" s="26" t="s">
+        <v>535</v>
+      </c>
+      <c r="G199" s="26" t="s">
+        <v>536</v>
+      </c>
+      <c r="H199" s="26">
+        <v>69</v>
+      </c>
+      <c r="I199" s="26">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="J199" s="26">
+        <v>60</v>
+      </c>
+      <c r="K199" s="28">
+        <v>0.34444444444444444</v>
+      </c>
+      <c r="L199" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M199" s="26">
+        <v>58</v>
+      </c>
+      <c r="N199" s="26" t="s">
+        <v>537</v>
+      </c>
+      <c r="P199" s="26">
+        <v>75</v>
+      </c>
+      <c r="Q199" s="26">
+        <v>92</v>
+      </c>
+      <c r="R199" s="26" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="200" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A200" s="26">
+        <v>250</v>
+      </c>
+      <c r="B200" s="27">
+        <v>46163</v>
+      </c>
+      <c r="C200" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D200" s="26" t="s">
+        <v>539</v>
+      </c>
+      <c r="E200" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F200" s="26" t="s">
+        <v>535</v>
+      </c>
+      <c r="G200" s="26" t="s">
+        <v>540</v>
+      </c>
+      <c r="H200" s="26">
+        <v>49</v>
+      </c>
+      <c r="I200" s="26">
+        <v>84.2</v>
+      </c>
+      <c r="J200" s="26">
+        <v>60</v>
+      </c>
+      <c r="K200" s="28">
+        <v>0.50138888888888888</v>
+      </c>
+      <c r="L200" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M200" s="26">
+        <v>63</v>
+      </c>
+      <c r="N200" s="26" t="s">
+        <v>541</v>
+      </c>
+      <c r="P200" s="26">
+        <v>70</v>
+      </c>
+      <c r="Q200" s="26">
+        <v>97</v>
+      </c>
+      <c r="R200" s="26" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="201" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A201" s="26">
+        <v>251</v>
+      </c>
+      <c r="B201" s="27">
+        <v>46163</v>
+      </c>
+      <c r="C201" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D201" s="26" t="s">
+        <v>543</v>
+      </c>
+      <c r="E201" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F201" s="26" t="s">
+        <v>544</v>
+      </c>
+      <c r="G201" s="26" t="s">
+        <v>545</v>
+      </c>
+      <c r="H201" s="26">
+        <v>30</v>
+      </c>
+      <c r="I201" s="26">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="J201" s="26">
+        <v>60</v>
+      </c>
+      <c r="K201" s="28">
+        <v>0.62222222222222223</v>
+      </c>
+      <c r="L201" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M201" s="26">
+        <v>61</v>
+      </c>
+      <c r="N201" s="26" t="s">
+        <v>546</v>
+      </c>
+      <c r="P201" s="26">
+        <v>73</v>
+      </c>
+      <c r="Q201" s="26">
+        <v>108</v>
+      </c>
+      <c r="R201" s="26" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="202" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A202" s="26">
+        <v>252</v>
+      </c>
+      <c r="B202" s="27">
+        <v>46164</v>
+      </c>
+      <c r="C202" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D202" s="26" t="s">
+        <v>553</v>
+      </c>
+      <c r="E202" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F202" s="26" t="s">
+        <v>554</v>
+      </c>
+      <c r="G202" s="26" t="s">
+        <v>555</v>
+      </c>
+      <c r="H202" s="26">
+        <v>85</v>
+      </c>
+      <c r="I202" s="26">
+        <v>77</v>
+      </c>
+      <c r="J202" s="26">
+        <v>30</v>
+      </c>
+      <c r="K202" s="28">
+        <v>0.31666666666666665</v>
+      </c>
+      <c r="L202" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M202" s="26">
+        <v>41</v>
+      </c>
+      <c r="N202" s="26" t="s">
+        <v>548</v>
+      </c>
+      <c r="P202" s="26">
+        <v>76</v>
+      </c>
+      <c r="Q202" s="26">
+        <v>95</v>
+      </c>
+      <c r="R202" s="26" t="s">
+        <v>556</v>
       </c>
     </row>
   </sheetData>
@@ -14995,7 +15932,7 @@
         <v>436837</v>
       </c>
       <c r="R88" s="3" t="s">
-        <v>480</v>
+        <v>549</v>
       </c>
     </row>
     <row r="89" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -15009,7 +15946,7 @@
         <v>224</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>481</v>
+        <v>550</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>179</v>
@@ -15324,7 +16261,7 @@
         <v>436837</v>
       </c>
       <c r="R95" s="3" t="s">
-        <v>482</v>
+        <v>551</v>
       </c>
     </row>
     <row r="96" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -15982,7 +16919,7 @@
         <v>352545</v>
       </c>
       <c r="R109" s="3" t="s">
-        <v>483</v>
+        <v>552</v>
       </c>
     </row>
     <row r="110" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
komodo Added: - Activities.bak.csv - komodo-dive-map.jpg Modified: - .gitignore - Activities (1).csv - Format.xlsm - Scuba_Log.xlsx - dive_script.py
</commit_message>
<xml_diff>
--- a/Scuba_Log.xlsx
+++ b/Scuba_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Akseldkw/Desktop/Aksel/Diving/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AE7D01-8ECE-0B45-BEC7-67A278813DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3A0D19-299D-024B-B443-887B6846EE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3360" yWindow="760" windowWidth="28460" windowHeight="23780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2740" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2772" uniqueCount="572">
   <si>
     <t>Dive Number</t>
   </si>
@@ -1667,9 +1667,33 @@
     <t>Manta dive!! So many mantas, just unreal. Manta came very close to me. Saw a blacktip reef shark as well</t>
   </si>
   <si>
+    <t>Manta Alley</t>
+  </si>
+  <si>
+    <t>Early morning, sunny</t>
+  </si>
+  <si>
+    <t>Cold</t>
+  </si>
+  <si>
     <t>0 days 15:39:35</t>
   </si>
   <si>
+    <t>Manta dive p2. Water was much murkier and colder than the previous days. We dove down to a manta cleaning station, but were unable to see as many. The current was very strong. The water was cold enough to take my breath away for a few seconds after entering</t>
+  </si>
+  <si>
+    <t>0 days 06:56:59</t>
+  </si>
+  <si>
+    <t>0 days 15:27:59</t>
+  </si>
+  <si>
+    <t>0 days 02:29:24</t>
+  </si>
+  <si>
+    <t>0 days 02:38:21</t>
+  </si>
+  <si>
     <t xml:space="preserve">First Huracan dive. DM was named Eric, really great dive. Saw reef shark, tarpon, snapper, schools of fish. Drift dive, wall started at 30ft and continued into the abyss to ~200 ft. Shot 3 lionfish and missed 2 more, saw shark right after shooting lionfish which spooked me a bit. </t>
   </si>
   <si>
@@ -1682,16 +1706,37 @@
     <t>Wall dive, buddied with mom. Saw no lionfish again! 3 turtles, reef sharkkd</t>
   </si>
   <si>
-    <t>Manta Alley</t>
-  </si>
-  <si>
-    <t>Early morning, sunny</t>
-  </si>
-  <si>
-    <t>Cold</t>
-  </si>
-  <si>
-    <t>Manta dive p2. Water was much murkier and colder than the previous days. We dove down to a manta cleaning station, but were unable to see as many. The current was very strong. The water was cold enough to take my breath away for a few seconds after entering</t>
+    <t>Pretty boring, went deep into sand. Was murky and visibility was low. At the end, the dive impoved a ton, and saw some very cool rock formations in the shallow water</t>
+  </si>
+  <si>
+    <t>Batu Balong</t>
+  </si>
+  <si>
+    <t>Cold at depth, warmer at top</t>
+  </si>
+  <si>
+    <t>Cool, strong currents</t>
+  </si>
+  <si>
+    <t>Very cool dive. This is a pinnacle jutting out from the bottom. The current was super strong, and flipped suddenly with the tide. Tons of schooling reef fish, Grand Trevally, turtle</t>
+  </si>
+  <si>
+    <t>Secret Garden</t>
+  </si>
+  <si>
+    <t>Tatawa Kecil</t>
+  </si>
+  <si>
+    <t>Siaba Kecil</t>
+  </si>
+  <si>
+    <t>Dropped into front of island (facing the current). Hooked in with reef hooks for 10 minutes or so. Then swam away from island towards deeper water, and got flushed by current to the backside of the island. I got yelled at for staying hooked in too long</t>
+  </si>
+  <si>
+    <t>Moderate current</t>
+  </si>
+  <si>
+    <t>Mom Angela and I drifted for a while. Very cool, saw shark, finished on the shallow reef. Got some cool videos of turtle feeding</t>
   </si>
 </sst>
 </file>
@@ -2156,7 +2201,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S202"/>
+  <dimension ref="A1:S206"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" customWidth="1"/>
@@ -11144,7 +11189,7 @@
     </row>
     <row r="189" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A189" s="26">
-        <v>220</v>
+        <v>188</v>
       </c>
       <c r="B189" s="27">
         <v>46159</v>
@@ -11197,7 +11242,7 @@
     </row>
     <row r="190" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A190" s="26">
-        <v>221</v>
+        <v>189</v>
       </c>
       <c r="B190" s="27">
         <v>46159</v>
@@ -11250,7 +11295,7 @@
     </row>
     <row r="191" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A191" s="26">
-        <v>223</v>
+        <v>190</v>
       </c>
       <c r="B191" s="27">
         <v>46160</v>
@@ -11303,7 +11348,7 @@
     </row>
     <row r="192" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A192" s="26">
-        <v>224</v>
+        <v>191</v>
       </c>
       <c r="B192" s="27">
         <v>46160</v>
@@ -11350,7 +11395,7 @@
     </row>
     <row r="193" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A193" s="26">
-        <v>225</v>
+        <v>192</v>
       </c>
       <c r="B193" s="27">
         <v>46160</v>
@@ -11400,7 +11445,7 @@
     </row>
     <row r="194" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A194" s="26">
-        <v>226</v>
+        <v>193</v>
       </c>
       <c r="B194" s="27">
         <v>46161</v>
@@ -11453,7 +11498,7 @@
     </row>
     <row r="195" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A195" s="26">
-        <v>227</v>
+        <v>194</v>
       </c>
       <c r="B195" s="27">
         <v>46161</v>
@@ -11506,7 +11551,7 @@
     </row>
     <row r="196" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A196" s="26">
-        <v>228</v>
+        <v>195</v>
       </c>
       <c r="B196" s="27">
         <v>46162</v>
@@ -11559,7 +11604,7 @@
     </row>
     <row r="197" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A197" s="26">
-        <v>247</v>
+        <v>196</v>
       </c>
       <c r="B197" s="27">
         <v>46162</v>
@@ -11612,7 +11657,7 @@
     </row>
     <row r="198" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A198" s="26">
-        <v>248</v>
+        <v>197</v>
       </c>
       <c r="B198" s="27">
         <v>46162</v>
@@ -11662,7 +11707,7 @@
     </row>
     <row r="199" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A199" s="26">
-        <v>249</v>
+        <v>198</v>
       </c>
       <c r="B199" s="27">
         <v>46163</v>
@@ -11715,7 +11760,7 @@
     </row>
     <row r="200" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A200" s="26">
-        <v>250</v>
+        <v>199</v>
       </c>
       <c r="B200" s="27">
         <v>46163</v>
@@ -11768,7 +11813,7 @@
     </row>
     <row r="201" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A201" s="26">
-        <v>251</v>
+        <v>200</v>
       </c>
       <c r="B201" s="27">
         <v>46163</v>
@@ -11821,7 +11866,7 @@
     </row>
     <row r="202" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A202" s="26">
-        <v>252</v>
+        <v>201</v>
       </c>
       <c r="B202" s="27">
         <v>46164</v>
@@ -11830,16 +11875,16 @@
         <v>281</v>
       </c>
       <c r="D202" s="26" t="s">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="E202" s="26" t="s">
         <v>531</v>
       </c>
       <c r="F202" s="26" t="s">
-        <v>554</v>
+        <v>549</v>
       </c>
       <c r="G202" s="26" t="s">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="H202" s="26">
         <v>85</v>
@@ -11860,7 +11905,7 @@
         <v>41</v>
       </c>
       <c r="N202" s="26" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="P202" s="26">
         <v>76</v>
@@ -11869,7 +11914,219 @@
         <v>95</v>
       </c>
       <c r="R202" s="26" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="203" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A203" s="26">
+        <v>202</v>
+      </c>
+      <c r="B203" s="27">
+        <v>46164</v>
+      </c>
+      <c r="C203" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D203" s="26" t="s">
+        <v>566</v>
+      </c>
+      <c r="E203" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F203" s="26" t="s">
+        <v>527</v>
+      </c>
+      <c r="G203" s="26" t="s">
+        <v>563</v>
+      </c>
+      <c r="H203" s="26">
+        <v>74</v>
+      </c>
+      <c r="I203" s="26">
+        <v>78.8</v>
+      </c>
+      <c r="J203" s="26">
+        <v>30</v>
+      </c>
+      <c r="K203" s="28">
+        <v>0.63402777777777775</v>
+      </c>
+      <c r="L203" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M203" s="26">
+        <v>56</v>
+      </c>
+      <c r="N203" s="26" t="s">
+        <v>553</v>
+      </c>
+      <c r="P203" s="26">
+        <v>72</v>
+      </c>
+      <c r="Q203" s="26">
+        <v>100</v>
+      </c>
+      <c r="R203" s="26" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="204" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A204" s="26">
+        <v>203</v>
+      </c>
+      <c r="B204" s="27">
+        <v>46165</v>
+      </c>
+      <c r="C204" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D204" s="26" t="s">
+        <v>562</v>
+      </c>
+      <c r="E204" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F204" s="26" t="s">
+        <v>549</v>
+      </c>
+      <c r="G204" s="26" t="s">
+        <v>564</v>
+      </c>
+      <c r="H204" s="26">
+        <v>82</v>
+      </c>
+      <c r="I204" s="26">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="J204" s="26">
+        <v>60</v>
+      </c>
+      <c r="K204" s="28">
+        <v>0.31666666666666665</v>
+      </c>
+      <c r="L204" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M204" s="26">
+        <v>60</v>
+      </c>
+      <c r="N204" s="26" t="s">
+        <v>554</v>
+      </c>
+      <c r="P204" s="26">
+        <v>64</v>
+      </c>
+      <c r="Q204" s="26">
+        <v>91</v>
+      </c>
+      <c r="R204" s="26" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="205" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A205" s="26">
+        <v>204</v>
+      </c>
+      <c r="B205" s="27">
+        <v>46165</v>
+      </c>
+      <c r="C205" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D205" s="26" t="s">
+        <v>567</v>
+      </c>
+      <c r="E205" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F205" s="26" t="s">
+        <v>527</v>
+      </c>
+      <c r="G205" s="26" t="s">
+        <v>500</v>
+      </c>
+      <c r="H205" s="26">
+        <v>100</v>
+      </c>
+      <c r="I205" s="26">
+        <v>84.2</v>
+      </c>
+      <c r="J205" s="26">
+        <v>60</v>
+      </c>
+      <c r="K205" s="28">
+        <v>0.46111111111111114</v>
+      </c>
+      <c r="L205" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M205" s="26">
+        <v>47</v>
+      </c>
+      <c r="N205" s="26" t="s">
+        <v>555</v>
+      </c>
+      <c r="P205" s="26">
+        <v>67</v>
+      </c>
+      <c r="Q205" s="26">
+        <v>88</v>
+      </c>
+      <c r="R205" s="26" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="206" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A206" s="26">
+        <v>205</v>
+      </c>
+      <c r="B206" s="27">
+        <v>46165</v>
+      </c>
+      <c r="C206" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D206" s="26" t="s">
+        <v>568</v>
+      </c>
+      <c r="E206" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F206" s="26" t="s">
+        <v>527</v>
+      </c>
+      <c r="G206" s="26" t="s">
+        <v>570</v>
+      </c>
+      <c r="H206" s="26">
+        <v>74</v>
+      </c>
+      <c r="I206" s="26">
+        <v>82.4</v>
+      </c>
+      <c r="J206" s="26">
+        <v>60</v>
+      </c>
+      <c r="K206" s="28">
+        <v>0.60277777777777775</v>
+      </c>
+      <c r="L206" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M206" s="26">
+        <v>62</v>
+      </c>
+      <c r="N206" s="26" t="s">
         <v>556</v>
+      </c>
+      <c r="P206" s="26">
+        <v>76</v>
+      </c>
+      <c r="Q206" s="26">
+        <v>99</v>
+      </c>
+      <c r="R206" s="26" t="s">
+        <v>571</v>
       </c>
     </row>
   </sheetData>
@@ -15932,7 +16189,7 @@
         <v>436837</v>
       </c>
       <c r="R88" s="3" t="s">
-        <v>549</v>
+        <v>557</v>
       </c>
     </row>
     <row r="89" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -15946,7 +16203,7 @@
         <v>224</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>550</v>
+        <v>558</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>179</v>
@@ -16261,7 +16518,7 @@
         <v>436837</v>
       </c>
       <c r="R95" s="3" t="s">
-        <v>551</v>
+        <v>559</v>
       </c>
     </row>
     <row r="96" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -16919,7 +17176,7 @@
         <v>352545</v>
       </c>
       <c r="R109" s="3" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
     </row>
     <row r="110" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
pictures-and-last-dives Added: - dive-map-lighthouse-reef-dive-belize.jpg - cozumel-dive-sites.jpg - cozumel-dive-sites.webp Modified: - Activities (1).csv - Activities.csv - Format.xlsm - Scuba_Log.xlsx
</commit_message>
<xml_diff>
--- a/Scuba_Log.xlsx
+++ b/Scuba_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Akseldkw/Desktop/Aksel/Diving/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3A0D19-299D-024B-B443-887B6846EE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5FF41E-3980-A44B-9AAA-F89EE93619E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="760" windowWidth="28460" windowHeight="23780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21640" yWindow="600" windowWidth="28460" windowHeight="23780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Log" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2772" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2804" uniqueCount="584">
   <si>
     <t>Dive Number</t>
   </si>
@@ -1625,9 +1625,6 @@
     <t>Best dive yet. Tons of fish, felt like a little fishtank. Mom accidentally knocked my watch off, and I lost it at the end of the dive (luckily recovered)</t>
   </si>
   <si>
-    <t>The Shotgun</t>
-  </si>
-  <si>
     <t>Warm, windy</t>
   </si>
   <si>
@@ -1682,18 +1679,63 @@
     <t>Manta dive p2. Water was much murkier and colder than the previous days. We dove down to a manta cleaning station, but were unable to see as many. The current was very strong. The water was cold enough to take my breath away for a few seconds after entering</t>
   </si>
   <si>
+    <t>Secret Garden</t>
+  </si>
+  <si>
+    <t>Cold at depth, warmer at top</t>
+  </si>
+  <si>
     <t>0 days 06:56:59</t>
   </si>
   <si>
+    <t>Pretty boring, went deep into sand. Was murky and visibility was low. At the end, the dive impoved a ton, and saw some very cool rock formations in the shallow water</t>
+  </si>
+  <si>
+    <t>Batu Balong</t>
+  </si>
+  <si>
+    <t>Cool, strong currents</t>
+  </si>
+  <si>
     <t>0 days 15:27:59</t>
   </si>
   <si>
+    <t>Very cool dive. This is a pinnacle jutting out from the bottom. The current was super strong, and flipped suddenly with the tide. Tons of schooling reef fish, Grand Trevally, turtle</t>
+  </si>
+  <si>
+    <t>Tatawa Kecil</t>
+  </si>
+  <si>
     <t>0 days 02:29:24</t>
   </si>
   <si>
+    <t>Dropped into front of island (facing the current). Hooked in with reef hooks for 10 minutes or so. Then swam away from island towards deeper water, and got flushed by current to the backside of the island. I got yelled at for staying hooked in too long</t>
+  </si>
+  <si>
+    <t>Siaba Kecil</t>
+  </si>
+  <si>
+    <t>Moderate current</t>
+  </si>
+  <si>
     <t>0 days 02:38:21</t>
   </si>
   <si>
+    <t>Mom Angela and I drifted for a while. Very cool, saw shark, finished on the shallow reef. Got some cool videos of turtle feeding</t>
+  </si>
+  <si>
+    <t>0 days 23:27:34</t>
+  </si>
+  <si>
+    <t>0 days 15:56:50</t>
+  </si>
+  <si>
+    <t>0 days 02:30:06</t>
+  </si>
+  <si>
+    <t>0 days 02:34:06</t>
+  </si>
+  <si>
     <t xml:space="preserve">First Huracan dive. DM was named Eric, really great dive. Saw reef shark, tarpon, snapper, schools of fish. Drift dive, wall started at 30ft and continued into the abyss to ~200 ft. Shot 3 lionfish and missed 2 more, saw shark right after shooting lionfish which spooked me a bit. </t>
   </si>
   <si>
@@ -1706,37 +1748,31 @@
     <t>Wall dive, buddied with mom. Saw no lionfish again! 3 turtles, reef sharkkd</t>
   </si>
   <si>
-    <t>Pretty boring, went deep into sand. Was murky and visibility was low. At the end, the dive impoved a ton, and saw some very cool rock formations in the shallow water</t>
-  </si>
-  <si>
-    <t>Batu Balong</t>
-  </si>
-  <si>
-    <t>Cold at depth, warmer at top</t>
-  </si>
-  <si>
-    <t>Cool, strong currents</t>
-  </si>
-  <si>
-    <t>Very cool dive. This is a pinnacle jutting out from the bottom. The current was super strong, and flipped suddenly with the tide. Tons of schooling reef fish, Grand Trevally, turtle</t>
-  </si>
-  <si>
-    <t>Secret Garden</t>
-  </si>
-  <si>
-    <t>Tatawa Kecil</t>
-  </si>
-  <si>
-    <t>Siaba Kecil</t>
-  </si>
-  <si>
-    <t>Dropped into front of island (facing the current). Hooked in with reef hooks for 10 minutes or so. Then swam away from island towards deeper water, and got flushed by current to the backside of the island. I got yelled at for staying hooked in too long</t>
-  </si>
-  <si>
-    <t>Moderate current</t>
-  </si>
-  <si>
-    <t>Mom Angela and I drifted for a while. Very cool, saw shark, finished on the shallow reef. Got some cool videos of turtle feeding</t>
+    <t>Shotgun</t>
+  </si>
+  <si>
+    <t>Castle Rock</t>
+  </si>
+  <si>
+    <t>Siaba Besar</t>
+  </si>
+  <si>
+    <t>Sunny &amp; windy</t>
+  </si>
+  <si>
+    <t>First dive post food-poisoning. Shallow reef, saw lots of cool stuff. Cute cuttlefish hung out with Laura and I for a few minutes. Saw sharks and huge Napolean Wrasse</t>
+  </si>
+  <si>
+    <t>Dropped into the front of the island. It was a little bit underwhelming at first, the visibility wasn't great. Saw sharks and jacks at a distance. Finished the dive using reef hooks with Benjy's group</t>
+  </si>
+  <si>
+    <t>Shotgun p2. The current was milder this time than the first time. It was super cool to see the reef at a slower pace. The highlights were the swimthroughs that we were able to explore due to the milder current. Saw some great corals, schooling Jacks, shark that got close</t>
+  </si>
+  <si>
+    <t>Crystall Rock was awesome, I preferred it to Castle Rock. Saw tons of jacks chasing baitfish, some juvenile sharks hiding under coral, enormous corals on the backside of the rock. Great dive to end the trip on.</t>
+  </si>
+  <si>
+    <t>Crystal Rock</t>
   </si>
 </sst>
 </file>
@@ -1876,6 +1912,143 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>172720</xdr:colOff>
+      <xdr:row>188</xdr:row>
+      <xdr:rowOff>71120</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>20320</xdr:colOff>
+      <xdr:row>206</xdr:row>
+      <xdr:rowOff>1206</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B20670F1-28FC-5BFE-933B-3E6BDE685DAF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="36596320" y="37470080"/>
+          <a:ext cx="3962400" cy="3587686"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>375920</xdr:colOff>
+      <xdr:row>151</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>518160</xdr:colOff>
+      <xdr:row>176</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93510163-5DBB-195C-6422-9C14EEEC4999}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="43383200" y="30002480"/>
+          <a:ext cx="5080000" cy="5080000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>-1</xdr:colOff>
+      <xdr:row>126</xdr:row>
+      <xdr:rowOff>138907</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>670791</xdr:colOff>
+      <xdr:row>150</xdr:row>
+      <xdr:rowOff>19845</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5832EBED-C72F-7AB7-A000-C3D6EECF905C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="36611718" y="25122188"/>
+          <a:ext cx="7338292" cy="4643438"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2201,7 +2374,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S206"/>
+  <dimension ref="A1:S210"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" customWidth="1"/>
@@ -11716,16 +11889,16 @@
         <v>281</v>
       </c>
       <c r="D199" s="26" t="s">
-        <v>534</v>
+        <v>575</v>
       </c>
       <c r="E199" s="26" t="s">
         <v>531</v>
       </c>
       <c r="F199" s="26" t="s">
+        <v>534</v>
+      </c>
+      <c r="G199" s="26" t="s">
         <v>535</v>
-      </c>
-      <c r="G199" s="26" t="s">
-        <v>536</v>
       </c>
       <c r="H199" s="26">
         <v>69</v>
@@ -11746,7 +11919,7 @@
         <v>58</v>
       </c>
       <c r="N199" s="26" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="P199" s="26">
         <v>75</v>
@@ -11755,7 +11928,7 @@
         <v>92</v>
       </c>
       <c r="R199" s="26" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="200" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -11769,16 +11942,16 @@
         <v>281</v>
       </c>
       <c r="D200" s="26" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E200" s="26" t="s">
         <v>531</v>
       </c>
       <c r="F200" s="26" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="G200" s="26" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="H200" s="26">
         <v>49</v>
@@ -11799,7 +11972,7 @@
         <v>63</v>
       </c>
       <c r="N200" s="26" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="P200" s="26">
         <v>70</v>
@@ -11808,7 +11981,7 @@
         <v>97</v>
       </c>
       <c r="R200" s="26" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="201" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -11822,16 +11995,16 @@
         <v>281</v>
       </c>
       <c r="D201" s="26" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="E201" s="26" t="s">
         <v>531</v>
       </c>
       <c r="F201" s="26" t="s">
+        <v>543</v>
+      </c>
+      <c r="G201" s="26" t="s">
         <v>544</v>
-      </c>
-      <c r="G201" s="26" t="s">
-        <v>545</v>
       </c>
       <c r="H201" s="26">
         <v>30</v>
@@ -11852,7 +12025,7 @@
         <v>61</v>
       </c>
       <c r="N201" s="26" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="P201" s="26">
         <v>73</v>
@@ -11861,7 +12034,7 @@
         <v>108</v>
       </c>
       <c r="R201" s="26" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="202" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -11875,16 +12048,16 @@
         <v>281</v>
       </c>
       <c r="D202" s="26" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E202" s="26" t="s">
         <v>531</v>
       </c>
       <c r="F202" s="26" t="s">
+        <v>548</v>
+      </c>
+      <c r="G202" s="26" t="s">
         <v>549</v>
-      </c>
-      <c r="G202" s="26" t="s">
-        <v>550</v>
       </c>
       <c r="H202" s="26">
         <v>85</v>
@@ -11905,7 +12078,7 @@
         <v>41</v>
       </c>
       <c r="N202" s="26" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="P202" s="26">
         <v>76</v>
@@ -11914,7 +12087,7 @@
         <v>95</v>
       </c>
       <c r="R202" s="26" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="203" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -11928,7 +12101,7 @@
         <v>281</v>
       </c>
       <c r="D203" s="26" t="s">
-        <v>566</v>
+        <v>552</v>
       </c>
       <c r="E203" s="26" t="s">
         <v>531</v>
@@ -11937,7 +12110,7 @@
         <v>527</v>
       </c>
       <c r="G203" s="26" t="s">
-        <v>563</v>
+        <v>553</v>
       </c>
       <c r="H203" s="26">
         <v>74</v>
@@ -11958,7 +12131,7 @@
         <v>56</v>
       </c>
       <c r="N203" s="26" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="P203" s="26">
         <v>72</v>
@@ -11967,7 +12140,7 @@
         <v>100</v>
       </c>
       <c r="R203" s="26" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
     </row>
     <row r="204" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -11981,16 +12154,16 @@
         <v>281</v>
       </c>
       <c r="D204" s="26" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="E204" s="26" t="s">
         <v>531</v>
       </c>
       <c r="F204" s="26" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="G204" s="26" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="H204" s="26">
         <v>82</v>
@@ -12011,7 +12184,7 @@
         <v>60</v>
       </c>
       <c r="N204" s="26" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="P204" s="26">
         <v>64</v>
@@ -12020,7 +12193,7 @@
         <v>91</v>
       </c>
       <c r="R204" s="26" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
     </row>
     <row r="205" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -12034,7 +12207,7 @@
         <v>281</v>
       </c>
       <c r="D205" s="26" t="s">
-        <v>567</v>
+        <v>560</v>
       </c>
       <c r="E205" s="26" t="s">
         <v>531</v>
@@ -12064,7 +12237,7 @@
         <v>47</v>
       </c>
       <c r="N205" s="26" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="P205" s="26">
         <v>67</v>
@@ -12073,7 +12246,7 @@
         <v>88</v>
       </c>
       <c r="R205" s="26" t="s">
-        <v>569</v>
+        <v>562</v>
       </c>
     </row>
     <row r="206" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
@@ -12087,7 +12260,7 @@
         <v>281</v>
       </c>
       <c r="D206" s="26" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="E206" s="26" t="s">
         <v>531</v>
@@ -12096,7 +12269,7 @@
         <v>527</v>
       </c>
       <c r="G206" s="26" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="H206" s="26">
         <v>74</v>
@@ -12117,7 +12290,7 @@
         <v>62</v>
       </c>
       <c r="N206" s="26" t="s">
-        <v>556</v>
+        <v>565</v>
       </c>
       <c r="P206" s="26">
         <v>76</v>
@@ -12126,11 +12299,224 @@
         <v>99</v>
       </c>
       <c r="R206" s="26" t="s">
-        <v>571</v>
+        <v>566</v>
+      </c>
+    </row>
+    <row r="207" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A207" s="26">
+        <v>206</v>
+      </c>
+      <c r="B207" s="27">
+        <v>46166</v>
+      </c>
+      <c r="C207" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D207" s="26" t="s">
+        <v>577</v>
+      </c>
+      <c r="E207" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F207" s="26" t="s">
+        <v>527</v>
+      </c>
+      <c r="G207" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="H207" s="26">
+        <v>77</v>
+      </c>
+      <c r="I207" s="26">
+        <v>84.2</v>
+      </c>
+      <c r="J207" s="26">
+        <v>80</v>
+      </c>
+      <c r="K207" s="28">
+        <v>0.62291666666666667</v>
+      </c>
+      <c r="L207" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M207" s="26">
+        <v>67</v>
+      </c>
+      <c r="N207" s="26" t="s">
+        <v>567</v>
+      </c>
+      <c r="P207" s="26">
+        <v>82</v>
+      </c>
+      <c r="Q207" s="26">
+        <v>110</v>
+      </c>
+      <c r="R207" s="26" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="208" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A208" s="26">
+        <v>207</v>
+      </c>
+      <c r="B208" s="27">
+        <v>46167</v>
+      </c>
+      <c r="C208" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D208" s="26" t="s">
+        <v>576</v>
+      </c>
+      <c r="E208" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F208" s="26" t="s">
+        <v>527</v>
+      </c>
+      <c r="G208" s="26" t="s">
+        <v>564</v>
+      </c>
+      <c r="H208" s="26">
+        <v>91</v>
+      </c>
+      <c r="I208" s="26">
+        <v>82.4</v>
+      </c>
+      <c r="J208" s="26">
+        <v>80</v>
+      </c>
+      <c r="K208" s="28">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="L208" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M208" s="26">
+        <v>59</v>
+      </c>
+      <c r="N208" s="26" t="s">
+        <v>568</v>
+      </c>
+      <c r="P208" s="26">
+        <v>73</v>
+      </c>
+      <c r="Q208" s="26">
+        <v>99</v>
+      </c>
+      <c r="R208" s="26" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="209" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A209" s="26">
+        <v>208</v>
+      </c>
+      <c r="B209" s="27">
+        <v>46167</v>
+      </c>
+      <c r="C209" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D209" s="26" t="s">
+        <v>575</v>
+      </c>
+      <c r="E209" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F209" s="26" t="s">
+        <v>578</v>
+      </c>
+      <c r="G209" s="26" t="s">
+        <v>564</v>
+      </c>
+      <c r="H209" s="26">
+        <v>69</v>
+      </c>
+      <c r="I209" s="26">
+        <v>86</v>
+      </c>
+      <c r="J209" s="26">
+        <v>80</v>
+      </c>
+      <c r="K209" s="28">
+        <v>0.4777777777777778</v>
+      </c>
+      <c r="L209" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M209" s="26">
+        <v>66</v>
+      </c>
+      <c r="N209" s="26" t="s">
+        <v>569</v>
+      </c>
+      <c r="P209" s="26">
+        <v>72</v>
+      </c>
+      <c r="Q209" s="26">
+        <v>103</v>
+      </c>
+      <c r="R209" s="26" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="210" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A210" s="26">
+        <v>209</v>
+      </c>
+      <c r="B210" s="27">
+        <v>46167</v>
+      </c>
+      <c r="C210" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="D210" s="26" t="s">
+        <v>583</v>
+      </c>
+      <c r="E210" s="26" t="s">
+        <v>531</v>
+      </c>
+      <c r="F210" s="26" t="s">
+        <v>578</v>
+      </c>
+      <c r="G210" s="26" t="s">
+        <v>564</v>
+      </c>
+      <c r="H210" s="26">
+        <v>82</v>
+      </c>
+      <c r="I210" s="26">
+        <v>82.4</v>
+      </c>
+      <c r="J210" s="26">
+        <v>80</v>
+      </c>
+      <c r="K210" s="28">
+        <v>0.62986111111111109</v>
+      </c>
+      <c r="L210" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="M210" s="26">
+        <v>63</v>
+      </c>
+      <c r="N210" s="26" t="s">
+        <v>570</v>
+      </c>
+      <c r="P210" s="26">
+        <v>75</v>
+      </c>
+      <c r="Q210" s="26">
+        <v>96</v>
+      </c>
+      <c r="R210" s="26" t="s">
+        <v>582</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -16189,7 +16575,7 @@
         <v>436837</v>
       </c>
       <c r="R88" s="3" t="s">
-        <v>557</v>
+        <v>571</v>
       </c>
     </row>
     <row r="89" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -16203,7 +16589,7 @@
         <v>224</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>558</v>
+        <v>572</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>179</v>
@@ -16518,7 +16904,7 @@
         <v>436837</v>
       </c>
       <c r="R95" s="3" t="s">
-        <v>559</v>
+        <v>573</v>
       </c>
     </row>
     <row r="96" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -17176,7 +17562,7 @@
         <v>352545</v>
       </c>
       <c r="R109" s="3" t="s">
-        <v>560</v>
+        <v>574</v>
       </c>
     </row>
     <row r="110" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>